<commit_message>
Últimos detalles y ajustes en gráficas
</commit_message>
<xml_diff>
--- a/TFG_Benchmark_Questions.xlsx
+++ b/TFG_Benchmark_Questions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Florian\Desktop\TFG_benchmark\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EF40348-69E4-4E26-A23E-327390F3341A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16258370-9D02-45C3-B13C-72F334D5D00F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1137,6 +1137,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
+  <numFmts count="1">
+    <numFmt numFmtId="169" formatCode="#,##0.000"/>
+  </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
@@ -1185,32 +1188,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="16">
-    <dxf>
-      <border>
-        <left style="thin">
-          <color rgb="FF356854"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF356854"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF356854"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF356854"/>
-        </bottom>
-      </border>
-    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1355,31 +1343,47 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color rgb="FF356854"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF356854"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF356854"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF356854"/>
+        </bottom>
+      </border>
+    </dxf>
   </dxfs>
   <tableStyles count="4" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="Arch1-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="12"/>
-      <tableStyleElement type="headerRow" dxfId="15"/>
-      <tableStyleElement type="firstRowStripe" dxfId="14"/>
-      <tableStyleElement type="secondRowStripe" dxfId="13"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="15"/>
+      <tableStyleElement type="headerRow" dxfId="14"/>
+      <tableStyleElement type="firstRowStripe" dxfId="13"/>
+      <tableStyleElement type="secondRowStripe" dxfId="12"/>
     </tableStyle>
     <tableStyle name="Arch2-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF01000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="8"/>
-      <tableStyleElement type="headerRow" dxfId="11"/>
-      <tableStyleElement type="firstRowStripe" dxfId="10"/>
-      <tableStyleElement type="secondRowStripe" dxfId="9"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="11"/>
+      <tableStyleElement type="headerRow" dxfId="10"/>
+      <tableStyleElement type="firstRowStripe" dxfId="9"/>
+      <tableStyleElement type="secondRowStripe" dxfId="8"/>
     </tableStyle>
     <tableStyle name="Arch3-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF02000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="4"/>
-      <tableStyleElement type="headerRow" dxfId="7"/>
-      <tableStyleElement type="firstRowStripe" dxfId="6"/>
-      <tableStyleElement type="secondRowStripe" dxfId="5"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="7"/>
+      <tableStyleElement type="headerRow" dxfId="6"/>
+      <tableStyleElement type="firstRowStripe" dxfId="5"/>
+      <tableStyleElement type="secondRowStripe" dxfId="4"/>
     </tableStyle>
     <tableStyle name="Costes_Tokens-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF03000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="0"/>
-      <tableStyleElement type="headerRow" dxfId="3"/>
-      <tableStyleElement type="firstRowStripe" dxfId="2"/>
-      <tableStyleElement type="secondRowStripe" dxfId="1"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="3"/>
+      <tableStyleElement type="headerRow" dxfId="2"/>
+      <tableStyleElement type="firstRowStripe" dxfId="1"/>
+      <tableStyleElement type="secondRowStripe" dxfId="0"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -1593,6 +1597,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:P21"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="6" max="6" width="24.42578125" customWidth="1"/>
+    <col min="7" max="7" width="20.28515625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
@@ -1663,7 +1671,8 @@
       <c r="F2">
         <v>13011</v>
       </c>
-      <c r="G2">
+      <c r="G2" s="2">
+        <f>F2/1000</f>
         <v>13.010999999999999</v>
       </c>
       <c r="H2">
@@ -1713,7 +1722,8 @@
       <c r="F3">
         <v>5518</v>
       </c>
-      <c r="G3">
+      <c r="G3" s="2">
+        <f>F3/1000</f>
         <v>5.5179999999999998</v>
       </c>
       <c r="H3">
@@ -1763,7 +1773,8 @@
       <c r="F4">
         <v>9095</v>
       </c>
-      <c r="G4">
+      <c r="G4" s="2">
+        <f t="shared" ref="G3:G21" si="0">F4/1000</f>
         <v>9.0950000000000006</v>
       </c>
       <c r="H4">
@@ -1813,7 +1824,8 @@
       <c r="F5">
         <v>9173</v>
       </c>
-      <c r="G5">
+      <c r="G5" s="2">
+        <f t="shared" si="0"/>
         <v>9.173</v>
       </c>
       <c r="H5">
@@ -1863,7 +1875,8 @@
       <c r="F6">
         <v>9340</v>
       </c>
-      <c r="G6">
+      <c r="G6" s="2">
+        <f t="shared" si="0"/>
         <v>9.34</v>
       </c>
       <c r="H6">
@@ -1913,7 +1926,8 @@
       <c r="F7">
         <v>5205</v>
       </c>
-      <c r="G7">
+      <c r="G7" s="2">
+        <f t="shared" si="0"/>
         <v>5.2050000000000001</v>
       </c>
       <c r="H7">
@@ -1963,7 +1977,8 @@
       <c r="F8">
         <v>18708</v>
       </c>
-      <c r="G8">
+      <c r="G8" s="2">
+        <f t="shared" si="0"/>
         <v>18.707999999999998</v>
       </c>
       <c r="H8">
@@ -2013,7 +2028,8 @@
       <c r="F9">
         <v>4417</v>
       </c>
-      <c r="G9">
+      <c r="G9" s="2">
+        <f t="shared" si="0"/>
         <v>4.4169999999999998</v>
       </c>
       <c r="H9">
@@ -2063,7 +2079,8 @@
       <c r="F10">
         <v>7188</v>
       </c>
-      <c r="G10">
+      <c r="G10" s="2">
+        <f t="shared" si="0"/>
         <v>7.1879999999999997</v>
       </c>
       <c r="H10">
@@ -2113,7 +2130,8 @@
       <c r="F11">
         <v>15571</v>
       </c>
-      <c r="G11">
+      <c r="G11" s="2">
+        <f t="shared" si="0"/>
         <v>15.571</v>
       </c>
       <c r="H11">
@@ -2163,7 +2181,8 @@
       <c r="F12">
         <v>7075</v>
       </c>
-      <c r="G12">
+      <c r="G12" s="2">
+        <f t="shared" si="0"/>
         <v>7.0750000000000002</v>
       </c>
       <c r="H12">
@@ -2213,7 +2232,8 @@
       <c r="F13">
         <v>14498</v>
       </c>
-      <c r="G13">
+      <c r="G13" s="2">
+        <f t="shared" si="0"/>
         <v>14.497999999999999</v>
       </c>
       <c r="H13">
@@ -2263,7 +2283,8 @@
       <c r="F14">
         <v>4778</v>
       </c>
-      <c r="G14">
+      <c r="G14" s="2">
+        <f t="shared" si="0"/>
         <v>4.7779999999999996</v>
       </c>
       <c r="H14">
@@ -2313,7 +2334,8 @@
       <c r="F15">
         <v>11158</v>
       </c>
-      <c r="G15">
+      <c r="G15" s="2">
+        <f t="shared" si="0"/>
         <v>11.157999999999999</v>
       </c>
       <c r="H15">
@@ -2363,7 +2385,8 @@
       <c r="F16">
         <v>12461</v>
       </c>
-      <c r="G16">
+      <c r="G16" s="2">
+        <f t="shared" si="0"/>
         <v>12.461</v>
       </c>
       <c r="H16">
@@ -2413,7 +2436,8 @@
       <c r="F17">
         <v>7494</v>
       </c>
-      <c r="G17">
+      <c r="G17" s="2">
+        <f t="shared" si="0"/>
         <v>7.4939999999999998</v>
       </c>
       <c r="H17">
@@ -2463,7 +2487,8 @@
       <c r="F18">
         <v>10595</v>
       </c>
-      <c r="G18">
+      <c r="G18" s="2">
+        <f t="shared" si="0"/>
         <v>10.595000000000001</v>
       </c>
       <c r="H18">
@@ -2513,7 +2538,8 @@
       <c r="F19">
         <v>7458</v>
       </c>
-      <c r="G19">
+      <c r="G19" s="2">
+        <f t="shared" si="0"/>
         <v>7.4580000000000002</v>
       </c>
       <c r="H19">
@@ -2563,7 +2589,8 @@
       <c r="F20">
         <v>7689</v>
       </c>
-      <c r="G20">
+      <c r="G20" s="2">
+        <f t="shared" si="0"/>
         <v>7.6890000000000001</v>
       </c>
       <c r="H20">
@@ -2613,7 +2640,8 @@
       <c r="F21">
         <v>9888</v>
       </c>
-      <c r="G21">
+      <c r="G21" s="2">
+        <f t="shared" si="0"/>
         <v>9.8879999999999999</v>
       </c>
       <c r="H21">
@@ -2653,6 +2681,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:P21"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="6" max="6" width="18.85546875" customWidth="1"/>
+    <col min="7" max="7" width="31.140625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
@@ -2724,6 +2756,7 @@
         <v>21517</v>
       </c>
       <c r="G2">
+        <f>F2/1000</f>
         <v>21.516999999999999</v>
       </c>
       <c r="H2">
@@ -2774,6 +2807,7 @@
         <v>4983</v>
       </c>
       <c r="G3">
+        <f t="shared" ref="G3:G21" si="0">F3/1000</f>
         <v>4.9829999999999997</v>
       </c>
       <c r="H3">
@@ -2824,6 +2858,7 @@
         <v>4985</v>
       </c>
       <c r="G4">
+        <f t="shared" si="0"/>
         <v>4.9850000000000003</v>
       </c>
       <c r="H4">
@@ -2874,6 +2909,7 @@
         <v>6865</v>
       </c>
       <c r="G5">
+        <f t="shared" si="0"/>
         <v>6.8650000000000002</v>
       </c>
       <c r="H5">
@@ -2924,6 +2960,7 @@
         <v>3842</v>
       </c>
       <c r="G6">
+        <f t="shared" si="0"/>
         <v>3.8420000000000001</v>
       </c>
       <c r="H6">
@@ -2974,6 +3011,7 @@
         <v>6400</v>
       </c>
       <c r="G7">
+        <f t="shared" si="0"/>
         <v>6.4</v>
       </c>
       <c r="H7">
@@ -3024,6 +3062,7 @@
         <v>8317</v>
       </c>
       <c r="G8">
+        <f t="shared" si="0"/>
         <v>8.3170000000000002</v>
       </c>
       <c r="H8">
@@ -3074,6 +3113,7 @@
         <v>7181</v>
       </c>
       <c r="G9">
+        <f t="shared" si="0"/>
         <v>7.181</v>
       </c>
       <c r="H9">
@@ -3124,6 +3164,7 @@
         <v>58984</v>
       </c>
       <c r="G10">
+        <f t="shared" si="0"/>
         <v>58.984000000000002</v>
       </c>
       <c r="H10">
@@ -3174,6 +3215,7 @@
         <v>8393</v>
       </c>
       <c r="G11">
+        <f t="shared" si="0"/>
         <v>8.3930000000000007</v>
       </c>
       <c r="H11">
@@ -3224,6 +3266,7 @@
         <v>12831</v>
       </c>
       <c r="G12">
+        <f t="shared" si="0"/>
         <v>12.831</v>
       </c>
       <c r="H12">
@@ -3274,6 +3317,7 @@
         <v>11779</v>
       </c>
       <c r="G13">
+        <f t="shared" si="0"/>
         <v>11.779</v>
       </c>
       <c r="H13">
@@ -3324,6 +3368,7 @@
         <v>4450</v>
       </c>
       <c r="G14">
+        <f t="shared" si="0"/>
         <v>4.45</v>
       </c>
       <c r="H14">
@@ -3374,6 +3419,7 @@
         <v>16751</v>
       </c>
       <c r="G15">
+        <f t="shared" si="0"/>
         <v>16.751000000000001</v>
       </c>
       <c r="H15">
@@ -3424,6 +3470,7 @@
         <v>60144</v>
       </c>
       <c r="G16">
+        <f t="shared" si="0"/>
         <v>60.143999999999998</v>
       </c>
       <c r="H16">
@@ -3474,6 +3521,7 @@
         <v>7213</v>
       </c>
       <c r="G17">
+        <f t="shared" si="0"/>
         <v>7.2130000000000001</v>
       </c>
       <c r="H17">
@@ -3524,6 +3572,7 @@
         <v>53423</v>
       </c>
       <c r="G18">
+        <f t="shared" si="0"/>
         <v>53.423000000000002</v>
       </c>
       <c r="H18">
@@ -3574,6 +3623,7 @@
         <v>55314</v>
       </c>
       <c r="G19">
+        <f t="shared" si="0"/>
         <v>55.314</v>
       </c>
       <c r="H19">
@@ -3624,6 +3674,7 @@
         <v>147511</v>
       </c>
       <c r="G20">
+        <f t="shared" si="0"/>
         <v>147.511</v>
       </c>
       <c r="H20">
@@ -3674,6 +3725,7 @@
         <v>4692</v>
       </c>
       <c r="G21">
+        <f t="shared" si="0"/>
         <v>4.6920000000000002</v>
       </c>
       <c r="H21">
@@ -3713,6 +3765,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:Q21"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="6" max="6" width="19.7109375" customWidth="1"/>
+    <col min="7" max="7" width="22.28515625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
@@ -3787,6 +3843,7 @@
         <v>7108</v>
       </c>
       <c r="G2">
+        <f>F2/1000</f>
         <v>7.1079999999999997</v>
       </c>
       <c r="H2">
@@ -3840,6 +3897,7 @@
         <v>7113</v>
       </c>
       <c r="G3">
+        <f t="shared" ref="G3:G21" si="0">F3/1000</f>
         <v>7.1130000000000004</v>
       </c>
       <c r="H3">
@@ -3893,6 +3951,7 @@
         <v>5551</v>
       </c>
       <c r="G4">
+        <f t="shared" si="0"/>
         <v>5.5510000000000002</v>
       </c>
       <c r="H4">
@@ -3946,6 +4005,7 @@
         <v>9212</v>
       </c>
       <c r="G5">
+        <f t="shared" si="0"/>
         <v>9.2119999999999997</v>
       </c>
       <c r="H5">
@@ -3999,6 +4059,7 @@
         <v>8375</v>
       </c>
       <c r="G6">
+        <f t="shared" si="0"/>
         <v>8.375</v>
       </c>
       <c r="H6">
@@ -4052,6 +4113,7 @@
         <v>9057</v>
       </c>
       <c r="G7">
+        <f t="shared" si="0"/>
         <v>9.0570000000000004</v>
       </c>
       <c r="H7">
@@ -4105,6 +4167,7 @@
         <v>6598</v>
       </c>
       <c r="G8">
+        <f t="shared" si="0"/>
         <v>6.5979999999999999</v>
       </c>
       <c r="H8">
@@ -4158,6 +4221,7 @@
         <v>4623</v>
       </c>
       <c r="G9">
+        <f t="shared" si="0"/>
         <v>4.6230000000000002</v>
       </c>
       <c r="H9">
@@ -4211,6 +4275,7 @@
         <v>12280</v>
       </c>
       <c r="G10">
+        <f t="shared" si="0"/>
         <v>12.28</v>
       </c>
       <c r="H10">
@@ -4264,6 +4329,7 @@
         <v>7635</v>
       </c>
       <c r="G11">
+        <f t="shared" si="0"/>
         <v>7.6349999999999998</v>
       </c>
       <c r="H11">
@@ -4317,6 +4383,7 @@
         <v>8483</v>
       </c>
       <c r="G12">
+        <f t="shared" si="0"/>
         <v>8.4830000000000005</v>
       </c>
       <c r="H12">
@@ -4370,6 +4437,7 @@
         <v>18614</v>
       </c>
       <c r="G13">
+        <f t="shared" si="0"/>
         <v>18.614000000000001</v>
       </c>
       <c r="H13">
@@ -4423,6 +4491,7 @@
         <v>6051</v>
       </c>
       <c r="G14">
+        <f t="shared" si="0"/>
         <v>6.0510000000000002</v>
       </c>
       <c r="H14">
@@ -4476,6 +4545,7 @@
         <v>8849</v>
       </c>
       <c r="G15">
+        <f t="shared" si="0"/>
         <v>8.8490000000000002</v>
       </c>
       <c r="H15">
@@ -4529,6 +4599,7 @@
         <v>8785</v>
       </c>
       <c r="G16">
+        <f t="shared" si="0"/>
         <v>8.7850000000000001</v>
       </c>
       <c r="H16">
@@ -4582,6 +4653,7 @@
         <v>10522</v>
       </c>
       <c r="G17">
+        <f t="shared" si="0"/>
         <v>10.522</v>
       </c>
       <c r="H17">
@@ -4635,6 +4707,7 @@
         <v>11106</v>
       </c>
       <c r="G18">
+        <f t="shared" si="0"/>
         <v>11.106</v>
       </c>
       <c r="H18">
@@ -4688,6 +4761,7 @@
         <v>7463</v>
       </c>
       <c r="G19">
+        <f t="shared" si="0"/>
         <v>7.4630000000000001</v>
       </c>
       <c r="H19">
@@ -4741,6 +4815,7 @@
         <v>12691</v>
       </c>
       <c r="G20">
+        <f t="shared" si="0"/>
         <v>12.691000000000001</v>
       </c>
       <c r="H20">
@@ -4794,6 +4869,7 @@
         <v>11097</v>
       </c>
       <c r="G21">
+        <f t="shared" si="0"/>
         <v>11.097</v>
       </c>
       <c r="H21">

</xml_diff>

<commit_message>
Datasets con 2 PDFs más Un PDF de 85 páginas (más denso, con índice). Un PDF de 142 páginas (sin índice, menos denso)
</commit_message>
<xml_diff>
--- a/TFG_Benchmark_Questions.xlsx
+++ b/TFG_Benchmark_Questions.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Florian\Desktop\TFG_benchmark\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16258370-9D02-45C3-B13C-72F334D5D00F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86B9CCE4-7535-4BA4-9B7F-96DF99E89F6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Arch1" sheetId="1" r:id="rId1"/>
-    <sheet name="Arch2" sheetId="2" r:id="rId2"/>
-    <sheet name="Arch3" sheetId="3" r:id="rId3"/>
+    <sheet name="RAG_Pinecone" sheetId="1" r:id="rId1"/>
+    <sheet name="RAG_Native" sheetId="2" r:id="rId2"/>
+    <sheet name="LongContext" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="529" uniqueCount="274">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="529" uniqueCount="250">
   <si>
     <t>ID</t>
   </si>
@@ -47,42 +47,6 @@
   </si>
   <si>
     <t>Reference_Answer</t>
-  </si>
-  <si>
-    <t>Arch1_Response</t>
-  </si>
-  <si>
-    <t>Arch1_Time</t>
-  </si>
-  <si>
-    <t>Arch1_Time_seconds</t>
-  </si>
-  <si>
-    <t>Arch1_Input_Tokens</t>
-  </si>
-  <si>
-    <t>Arch1_Output_Tokens</t>
-  </si>
-  <si>
-    <t>Arch1_Chunks:</t>
-  </si>
-  <si>
-    <t>Arch1_Cost_Gemini-3_0-Flash</t>
-  </si>
-  <si>
-    <t>Arch1_Question_score_(0/10)</t>
-  </si>
-  <si>
-    <t>Arch1_Context_Found_(Sí/No)</t>
-  </si>
-  <si>
-    <t>Arch1_Hallucination</t>
-  </si>
-  <si>
-    <t>Arch1_Question_score_Judge(0/10)</t>
-  </si>
-  <si>
-    <t>Arch1_Judge_Reasoning</t>
   </si>
   <si>
     <t>Easy</t>
@@ -590,42 +554,6 @@
     <t>La respuesta generada proporciona detalles técnicos específicos que no están en la respuesta real, como límites de mecanizado y requisitos de juntas, lo cual es incorrecto según las especificaciones de BMW para cabezas Valvetronic.</t>
   </si>
   <si>
-    <t>Arch2_Response</t>
-  </si>
-  <si>
-    <t>Arch2_Time</t>
-  </si>
-  <si>
-    <t>Arch2_Time_seconds</t>
-  </si>
-  <si>
-    <t>Arch2_Input_Tokens</t>
-  </si>
-  <si>
-    <t>Arch2_Output_Tokens</t>
-  </si>
-  <si>
-    <t>Arch2_Chunks:</t>
-  </si>
-  <si>
-    <t>Arch2_Cost_Gemini-3_0-Flash</t>
-  </si>
-  <si>
-    <t>Arch2_Question_score_(0/10)</t>
-  </si>
-  <si>
-    <t>Arch2_Context_Found_(Sí/No)</t>
-  </si>
-  <si>
-    <t>Arch2_Hallucination</t>
-  </si>
-  <si>
-    <t>Arch2_Question_score_Judge(0/10)</t>
-  </si>
-  <si>
-    <t>Arch2_Judge_Reasoning</t>
-  </si>
-  <si>
     <t>According to the provided manual, the specific numerical gap setting is not listed. Instead, the manual states that the gap should be set to the value given by the spark plug manufacturer. 
 Additionally, the manual notes the following regarding spark plug gaps:
 *   **Multi-electrode plugs:** The gap between the centre electrode and the earth electrodes cannot be adjusted.
@@ -860,45 +788,6 @@
     <t>La respuesta generada es incorrecta, ya que afirma que se puede maquinar el cabezal del cilindro del motor N42, mientras que la respuesta real indica que generalmente no se permite debido a cambios en la geometría. Además, proporciona un límite de remoción de material que no está respaldado por la respuesta real.</t>
   </si>
   <si>
-    <t>Arch3_Response</t>
-  </si>
-  <si>
-    <t>Arch3_Time</t>
-  </si>
-  <si>
-    <t>Arch3_Time_seconds</t>
-  </si>
-  <si>
-    <t>Arch3_Input_Tokens</t>
-  </si>
-  <si>
-    <t>Arch3_Input_Tokens_PDF</t>
-  </si>
-  <si>
-    <t>Arch3_Output_Tokens</t>
-  </si>
-  <si>
-    <t>Arch3_Chunks:</t>
-  </si>
-  <si>
-    <t>Arch3_Cost_Gemini-3_0-Flash</t>
-  </si>
-  <si>
-    <t>Arch3_Question_score_(0/10)</t>
-  </si>
-  <si>
-    <t>Arch3_Context_Found_(Sí/No)</t>
-  </si>
-  <si>
-    <t>Arch3_Hallucination</t>
-  </si>
-  <si>
-    <t>Arch3_Question_score_Judge(0/10)</t>
-  </si>
-  <si>
-    <t>Arch3_Judge_Reasoning</t>
-  </si>
-  <si>
     <t>According to the technical data found in the Maintenance (Section 020) and Ignition System (Section 120) chapters of the BMW E46 Workshop Manual, the spark plug gap settings are determined by the engine type and the specific plug design installed.
 For the M43 4-cylinder engine and the M52 TU and M54 6-cylinder engines using standard spark plugs, the electrode gap is specified as 0.7 mm (0.027 in) with a tolerance of plus 0.1 mm.
 The manual notes that for the majority of E46 production models equipped with High Power ignition systems, multi-electrode spark plugs are utilized. Specifically, for the NGK BKR6EQUP and Bosch FGR7DQP four-electrode plugs, the gap is pre-set by the manufacturer and is classified as non-adjustable. The manual explicitly states that these electrodes must not be bent or adjusted.
@@ -1132,13 +1021,52 @@
   <si>
     <t>La respuesta generada es precisa y proporciona detalles adicionales útiles sobre las especificaciones del motor N42, incluyendo la altura estándar y la tolerancia de fabricación, así como las razones técnicas para no permitir el mecanizado.</t>
   </si>
+  <si>
+    <t>Response</t>
+  </si>
+  <si>
+    <t>Time</t>
+  </si>
+  <si>
+    <t>Time_seconds</t>
+  </si>
+  <si>
+    <t>Input_Tokens</t>
+  </si>
+  <si>
+    <t>Input_Tokens_PDF</t>
+  </si>
+  <si>
+    <t>Output_Tokens</t>
+  </si>
+  <si>
+    <t>Cost_Gemini-3_0-Flash</t>
+  </si>
+  <si>
+    <t>Question_score_(0/10)</t>
+  </si>
+  <si>
+    <t>Context_Found_(Sí/No)</t>
+  </si>
+  <si>
+    <t>Hallucination</t>
+  </si>
+  <si>
+    <t>Question_score_Judge(0/10)</t>
+  </si>
+  <si>
+    <t>Judge_Reasoning</t>
+  </si>
+  <si>
+    <t>Chunks</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <numFmts count="1">
-    <numFmt numFmtId="169" formatCode="#,##0.000"/>
+    <numFmt numFmtId="164" formatCode="#,##0.000"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -1193,7 +1121,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1616,40 +1544,40 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>4</v>
+        <v>237</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>5</v>
+        <v>238</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>6</v>
+        <v>239</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>7</v>
+        <v>240</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>8</v>
+        <v>242</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>9</v>
+        <v>249</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>10</v>
+        <v>243</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>11</v>
+        <v>244</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>12</v>
+        <v>245</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>13</v>
+        <v>246</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>14</v>
+        <v>247</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>15</v>
+        <v>248</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.2">
@@ -1657,16 +1585,16 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="D2" t="s">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="E2" t="s">
-        <v>19</v>
+        <v>7</v>
       </c>
       <c r="F2">
         <v>13011</v>
@@ -1688,19 +1616,19 @@
         <v>1.9039743920000001E-3</v>
       </c>
       <c r="L2" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="M2" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="N2" t="s">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="O2">
         <v>6</v>
       </c>
       <c r="P2" t="s">
-        <v>23</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.2">
@@ -1708,16 +1636,16 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="C3" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="D3" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="E3" t="s">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="F3">
         <v>5518</v>
@@ -1739,19 +1667,19 @@
         <v>1.5220821039999999E-3</v>
       </c>
       <c r="L3" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="M3" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="N3" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="O3">
         <v>8</v>
       </c>
       <c r="P3" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.2">
@@ -1759,22 +1687,22 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="C4" t="s">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="D4" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="E4" t="s">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="F4">
         <v>9095</v>
       </c>
       <c r="G4" s="2">
-        <f t="shared" ref="G3:G21" si="0">F4/1000</f>
+        <f t="shared" ref="G4:G21" si="0">F4/1000</f>
         <v>9.0950000000000006</v>
       </c>
       <c r="H4">
@@ -1790,19 +1718,19 @@
         <v>1.275250456E-3</v>
       </c>
       <c r="L4" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="M4" t="s">
+        <v>9</v>
+      </c>
+      <c r="N4" t="s">
         <v>21</v>
       </c>
-      <c r="N4" t="s">
-        <v>33</v>
-      </c>
       <c r="O4">
         <v>8</v>
       </c>
       <c r="P4" t="s">
-        <v>34</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.2">
@@ -1810,16 +1738,16 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="C5" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="D5" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="E5" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="F5">
         <v>9173</v>
@@ -1841,19 +1769,19 @@
         <v>2.0767736360000001E-3</v>
       </c>
       <c r="L5" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="M5" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="N5" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="O5">
         <v>8</v>
       </c>
       <c r="P5" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.2">
@@ -1861,16 +1789,16 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" t="s">
         <v>29</v>
       </c>
-      <c r="C6" t="s">
-        <v>40</v>
-      </c>
-      <c r="D6" t="s">
-        <v>41</v>
-      </c>
       <c r="E6" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="F6">
         <v>9340</v>
@@ -1892,19 +1820,19 @@
         <v>1.39219834E-3</v>
       </c>
       <c r="L6" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="M6" t="s">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="N6" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="O6">
         <v>3</v>
       </c>
       <c r="P6" t="s">
-        <v>46</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.2">
@@ -1912,16 +1840,16 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="C7" t="s">
-        <v>47</v>
+        <v>35</v>
       </c>
       <c r="D7" t="s">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="E7" t="s">
-        <v>49</v>
+        <v>37</v>
       </c>
       <c r="F7">
         <v>5205</v>
@@ -1943,19 +1871,19 @@
         <v>1.6468615480000001E-3</v>
       </c>
       <c r="L7" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="M7" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="N7" t="s">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="O7">
         <v>9</v>
       </c>
       <c r="P7" t="s">
-        <v>51</v>
+        <v>39</v>
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.2">
@@ -1963,16 +1891,16 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>52</v>
+        <v>40</v>
       </c>
       <c r="C8" t="s">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="D8" t="s">
-        <v>54</v>
+        <v>42</v>
       </c>
       <c r="E8" t="s">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="F8">
         <v>18708</v>
@@ -1994,19 +1922,19 @@
         <v>1.9099128239999999E-3</v>
       </c>
       <c r="L8" t="s">
-        <v>56</v>
+        <v>44</v>
       </c>
       <c r="M8" t="s">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="N8" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="O8">
         <v>3</v>
       </c>
       <c r="P8" t="s">
-        <v>58</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.2">
@@ -2014,16 +1942,16 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>52</v>
+        <v>40</v>
       </c>
       <c r="C9" t="s">
-        <v>59</v>
+        <v>47</v>
       </c>
       <c r="D9" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="E9" t="s">
-        <v>61</v>
+        <v>49</v>
       </c>
       <c r="F9">
         <v>4417</v>
@@ -2045,19 +1973,19 @@
         <v>1.0043974959999999E-3</v>
       </c>
       <c r="L9" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="M9" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="N9" t="s">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="O9">
         <v>10</v>
       </c>
       <c r="P9" t="s">
-        <v>62</v>
+        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.2">
@@ -2065,16 +1993,16 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
+        <v>40</v>
+      </c>
+      <c r="C10" t="s">
+        <v>51</v>
+      </c>
+      <c r="D10" t="s">
         <v>52</v>
       </c>
-      <c r="C10" t="s">
-        <v>63</v>
-      </c>
-      <c r="D10" t="s">
-        <v>64</v>
-      </c>
       <c r="E10" t="s">
-        <v>65</v>
+        <v>53</v>
       </c>
       <c r="F10">
         <v>7188</v>
@@ -2096,19 +2024,19 @@
         <v>1.651390804E-3</v>
       </c>
       <c r="L10" t="s">
-        <v>66</v>
+        <v>54</v>
       </c>
       <c r="M10" t="s">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="N10" t="s">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="O10">
         <v>2</v>
       </c>
       <c r="P10" t="s">
-        <v>68</v>
+        <v>56</v>
       </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.2">
@@ -2116,16 +2044,16 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>52</v>
+        <v>40</v>
       </c>
       <c r="C11" t="s">
-        <v>69</v>
+        <v>57</v>
       </c>
       <c r="D11" t="s">
-        <v>70</v>
+        <v>58</v>
       </c>
       <c r="E11" t="s">
-        <v>71</v>
+        <v>59</v>
       </c>
       <c r="F11">
         <v>15571</v>
@@ -2147,19 +2075,19 @@
         <v>1.7628457959999999E-3</v>
       </c>
       <c r="L11" t="s">
-        <v>72</v>
+        <v>60</v>
       </c>
       <c r="M11" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="N11" t="s">
-        <v>73</v>
+        <v>61</v>
       </c>
       <c r="O11">
         <v>4</v>
       </c>
       <c r="P11" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.2">
@@ -2167,16 +2095,16 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>75</v>
+        <v>63</v>
       </c>
       <c r="C12" t="s">
-        <v>76</v>
+        <v>64</v>
       </c>
       <c r="D12" t="s">
-        <v>77</v>
+        <v>65</v>
       </c>
       <c r="E12" t="s">
-        <v>78</v>
+        <v>66</v>
       </c>
       <c r="F12">
         <v>7075</v>
@@ -2198,19 +2126,19 @@
         <v>1.397086292E-3</v>
       </c>
       <c r="L12" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="M12" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="N12" t="s">
-        <v>79</v>
+        <v>67</v>
       </c>
       <c r="O12">
         <v>10</v>
       </c>
       <c r="P12" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.2">
@@ -2218,16 +2146,16 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>75</v>
+        <v>63</v>
       </c>
       <c r="C13" t="s">
-        <v>81</v>
+        <v>69</v>
       </c>
       <c r="D13" t="s">
-        <v>82</v>
+        <v>70</v>
       </c>
       <c r="E13" t="s">
-        <v>83</v>
+        <v>71</v>
       </c>
       <c r="F13">
         <v>14498</v>
@@ -2249,19 +2177,19 @@
         <v>2.2847649839999999E-3</v>
       </c>
       <c r="L13" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="M13" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="N13" t="s">
-        <v>84</v>
+        <v>72</v>
       </c>
       <c r="O13">
         <v>9</v>
       </c>
       <c r="P13" t="s">
-        <v>85</v>
+        <v>73</v>
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.2">
@@ -2269,16 +2197,16 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
+        <v>63</v>
+      </c>
+      <c r="C14" t="s">
+        <v>74</v>
+      </c>
+      <c r="D14" t="s">
         <v>75</v>
       </c>
-      <c r="C14" t="s">
-        <v>86</v>
-      </c>
-      <c r="D14" t="s">
-        <v>87</v>
-      </c>
       <c r="E14" t="s">
-        <v>88</v>
+        <v>76</v>
       </c>
       <c r="F14">
         <v>4778</v>
@@ -2300,19 +2228,19 @@
         <v>1.397531832E-3</v>
       </c>
       <c r="L14" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="M14" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="N14" t="s">
-        <v>89</v>
+        <v>77</v>
       </c>
       <c r="O14">
         <v>10</v>
       </c>
       <c r="P14" t="s">
-        <v>90</v>
+        <v>78</v>
       </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.2">
@@ -2320,16 +2248,16 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>75</v>
+        <v>63</v>
       </c>
       <c r="C15" t="s">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="D15" t="s">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="E15" t="s">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="F15">
         <v>11158</v>
@@ -2351,19 +2279,19 @@
         <v>1.7389810999999999E-3</v>
       </c>
       <c r="L15" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="M15" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="N15" t="s">
-        <v>94</v>
+        <v>82</v>
       </c>
       <c r="O15">
         <v>8</v>
       </c>
       <c r="P15" t="s">
-        <v>95</v>
+        <v>83</v>
       </c>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.2">
@@ -2371,16 +2299,16 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>96</v>
+        <v>84</v>
       </c>
       <c r="C16" t="s">
-        <v>97</v>
+        <v>85</v>
       </c>
       <c r="D16" t="s">
-        <v>98</v>
+        <v>86</v>
       </c>
       <c r="E16" t="s">
-        <v>99</v>
+        <v>87</v>
       </c>
       <c r="F16">
         <v>12461</v>
@@ -2402,19 +2330,19 @@
         <v>1.5531065239999999E-3</v>
       </c>
       <c r="L16" t="s">
-        <v>66</v>
+        <v>54</v>
       </c>
       <c r="M16" t="s">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="N16" t="s">
-        <v>100</v>
+        <v>88</v>
       </c>
       <c r="O16">
         <v>6</v>
       </c>
       <c r="P16" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.2">
@@ -2422,16 +2350,16 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>96</v>
+        <v>84</v>
       </c>
       <c r="C17" t="s">
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="D17" t="s">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="E17" t="s">
-        <v>104</v>
+        <v>92</v>
       </c>
       <c r="F17">
         <v>7494</v>
@@ -2453,19 +2381,19 @@
         <v>1.537763688E-3</v>
       </c>
       <c r="L17" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="M17" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="N17" t="s">
-        <v>105</v>
+        <v>93</v>
       </c>
       <c r="O17">
         <v>5</v>
       </c>
       <c r="P17" t="s">
-        <v>106</v>
+        <v>94</v>
       </c>
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.2">
@@ -2473,16 +2401,16 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
+        <v>84</v>
+      </c>
+      <c r="C18" t="s">
+        <v>95</v>
+      </c>
+      <c r="D18" t="s">
         <v>96</v>
       </c>
-      <c r="C18" t="s">
-        <v>107</v>
-      </c>
-      <c r="D18" t="s">
-        <v>108</v>
-      </c>
       <c r="E18" t="s">
-        <v>109</v>
+        <v>97</v>
       </c>
       <c r="F18">
         <v>10595</v>
@@ -2504,19 +2432,19 @@
         <v>2.732789828E-3</v>
       </c>
       <c r="L18" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="M18" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="N18" t="s">
-        <v>110</v>
+        <v>98</v>
       </c>
       <c r="O18">
         <v>8</v>
       </c>
       <c r="P18" t="s">
-        <v>111</v>
+        <v>99</v>
       </c>
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.2">
@@ -2524,16 +2452,16 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>96</v>
+        <v>84</v>
       </c>
       <c r="C19" t="s">
-        <v>112</v>
+        <v>100</v>
       </c>
       <c r="D19" t="s">
-        <v>113</v>
+        <v>101</v>
       </c>
       <c r="E19" t="s">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="F19">
         <v>7458</v>
@@ -2555,19 +2483,19 @@
         <v>1.8456363759999999E-3</v>
       </c>
       <c r="L19" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="M19" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="N19" t="s">
-        <v>115</v>
+        <v>103</v>
       </c>
       <c r="O19">
         <v>8</v>
       </c>
       <c r="P19" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.2">
@@ -2575,16 +2503,16 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>117</v>
+        <v>105</v>
       </c>
       <c r="C20" t="s">
-        <v>118</v>
+        <v>106</v>
       </c>
       <c r="D20" t="s">
-        <v>119</v>
+        <v>107</v>
       </c>
       <c r="E20" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="F20">
         <v>7689</v>
@@ -2606,19 +2534,19 @@
         <v>1.7125115440000001E-3</v>
       </c>
       <c r="L20" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="M20" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="N20" t="s">
-        <v>122</v>
+        <v>110</v>
       </c>
       <c r="O20">
         <v>8</v>
       </c>
       <c r="P20" t="s">
-        <v>123</v>
+        <v>111</v>
       </c>
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.2">
@@ -2626,16 +2554,16 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>117</v>
+        <v>105</v>
       </c>
       <c r="C21" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
       <c r="D21" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="E21" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="F21">
         <v>9888</v>
@@ -2657,19 +2585,19 @@
         <v>1.9188546159999999E-3</v>
       </c>
       <c r="L21" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="M21" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="N21" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="O21">
         <v>3</v>
       </c>
       <c r="P21" t="s">
-        <v>128</v>
+        <v>116</v>
       </c>
     </row>
   </sheetData>
@@ -2700,40 +2628,40 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>129</v>
+        <v>237</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>130</v>
+        <v>238</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>131</v>
+        <v>239</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>132</v>
+        <v>240</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>133</v>
+        <v>242</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>134</v>
+        <v>249</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>135</v>
+        <v>243</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>136</v>
+        <v>244</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>137</v>
+        <v>245</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>138</v>
+        <v>246</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>139</v>
+        <v>247</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>140</v>
+        <v>248</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.2">
@@ -2741,16 +2669,16 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="D2" t="s">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="E2" t="s">
-        <v>141</v>
+        <v>117</v>
       </c>
       <c r="F2">
         <v>21517</v>
@@ -2772,19 +2700,19 @@
         <v>1.2422727289999999E-2</v>
       </c>
       <c r="L2" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="M2" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="N2" t="s">
-        <v>142</v>
+        <v>118</v>
       </c>
       <c r="O2">
         <v>3</v>
       </c>
       <c r="P2" t="s">
-        <v>143</v>
+        <v>119</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.2">
@@ -2792,16 +2720,16 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="C3" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="D3" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="E3" t="s">
-        <v>144</v>
+        <v>120</v>
       </c>
       <c r="F3">
         <v>4983</v>
@@ -2823,19 +2751,19 @@
         <v>1.042745466E-2</v>
       </c>
       <c r="L3" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="M3" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="N3" t="s">
-        <v>145</v>
+        <v>121</v>
       </c>
       <c r="O3">
         <v>8</v>
       </c>
       <c r="P3" t="s">
-        <v>146</v>
+        <v>122</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.2">
@@ -2843,16 +2771,16 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="C4" t="s">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="D4" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="E4" t="s">
-        <v>147</v>
+        <v>123</v>
       </c>
       <c r="F4">
         <v>4985</v>
@@ -2874,19 +2802,19 @@
         <v>1.337145296E-2</v>
       </c>
       <c r="L4" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="M4" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="N4" t="s">
-        <v>148</v>
+        <v>124</v>
       </c>
       <c r="O4">
         <v>9</v>
       </c>
       <c r="P4" t="s">
-        <v>149</v>
+        <v>125</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.2">
@@ -2894,16 +2822,16 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="C5" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="D5" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="E5" t="s">
-        <v>150</v>
+        <v>126</v>
       </c>
       <c r="F5">
         <v>6865</v>
@@ -2925,19 +2853,19 @@
         <v>1.2954526480000001E-2</v>
       </c>
       <c r="L5" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="M5" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="N5" t="s">
-        <v>151</v>
+        <v>127</v>
       </c>
       <c r="O5">
         <v>8</v>
       </c>
       <c r="P5" t="s">
-        <v>152</v>
+        <v>128</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.2">
@@ -2945,16 +2873,16 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" t="s">
         <v>29</v>
       </c>
-      <c r="C6" t="s">
-        <v>40</v>
-      </c>
-      <c r="D6" t="s">
-        <v>41</v>
-      </c>
       <c r="E6" t="s">
-        <v>153</v>
+        <v>129</v>
       </c>
       <c r="F6">
         <v>3842</v>
@@ -2976,19 +2904,19 @@
         <v>1.1065120479999999E-2</v>
       </c>
       <c r="L6" t="s">
-        <v>72</v>
+        <v>60</v>
       </c>
       <c r="M6" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="N6" t="s">
-        <v>154</v>
+        <v>130</v>
       </c>
       <c r="O6">
         <v>8</v>
       </c>
       <c r="P6" t="s">
-        <v>155</v>
+        <v>131</v>
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.2">
@@ -2996,16 +2924,16 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="C7" t="s">
-        <v>47</v>
+        <v>35</v>
       </c>
       <c r="D7" t="s">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="E7" t="s">
-        <v>156</v>
+        <v>132</v>
       </c>
       <c r="F7">
         <v>6400</v>
@@ -3027,19 +2955,19 @@
         <v>1.287052315E-2</v>
       </c>
       <c r="L7" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="M7" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="N7" t="s">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="O7">
         <v>8</v>
       </c>
       <c r="P7" t="s">
-        <v>157</v>
+        <v>133</v>
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.2">
@@ -3047,16 +2975,16 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>52</v>
+        <v>40</v>
       </c>
       <c r="C8" t="s">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="D8" t="s">
-        <v>54</v>
+        <v>42</v>
       </c>
       <c r="E8" t="s">
-        <v>158</v>
+        <v>134</v>
       </c>
       <c r="F8">
         <v>8317</v>
@@ -3078,19 +3006,19 @@
         <v>1.9366467809999999E-2</v>
       </c>
       <c r="L8" t="s">
-        <v>56</v>
+        <v>44</v>
       </c>
       <c r="M8" t="s">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="N8" t="s">
-        <v>159</v>
+        <v>135</v>
       </c>
       <c r="O8">
         <v>3</v>
       </c>
       <c r="P8" t="s">
-        <v>160</v>
+        <v>136</v>
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.2">
@@ -3098,16 +3026,16 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>52</v>
+        <v>40</v>
       </c>
       <c r="C9" t="s">
-        <v>59</v>
+        <v>47</v>
       </c>
       <c r="D9" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="E9" t="s">
-        <v>161</v>
+        <v>137</v>
       </c>
       <c r="F9">
         <v>7181</v>
@@ -3129,19 +3057,19 @@
         <v>1.264128041E-2</v>
       </c>
       <c r="L9" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="M9" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="N9" t="s">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="O9">
         <v>10</v>
       </c>
       <c r="P9" t="s">
-        <v>162</v>
+        <v>138</v>
       </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.2">
@@ -3149,16 +3077,16 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
+        <v>40</v>
+      </c>
+      <c r="C10" t="s">
+        <v>51</v>
+      </c>
+      <c r="D10" t="s">
         <v>52</v>
       </c>
-      <c r="C10" t="s">
-        <v>63</v>
-      </c>
-      <c r="D10" t="s">
-        <v>64</v>
-      </c>
       <c r="E10" t="s">
-        <v>163</v>
+        <v>139</v>
       </c>
       <c r="F10">
         <v>58984</v>
@@ -3180,19 +3108,19 @@
         <v>1.534754659E-2</v>
       </c>
       <c r="L10" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="M10" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="N10" t="s">
-        <v>164</v>
+        <v>140</v>
       </c>
       <c r="O10">
         <v>2</v>
       </c>
       <c r="P10" t="s">
-        <v>165</v>
+        <v>141</v>
       </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.2">
@@ -3200,16 +3128,16 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>52</v>
+        <v>40</v>
       </c>
       <c r="C11" t="s">
-        <v>69</v>
+        <v>57</v>
       </c>
       <c r="D11" t="s">
-        <v>70</v>
+        <v>58</v>
       </c>
       <c r="E11" t="s">
-        <v>166</v>
+        <v>142</v>
       </c>
       <c r="F11">
         <v>8393</v>
@@ -3231,19 +3159,19 @@
         <v>1.696123469E-2</v>
       </c>
       <c r="L11" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="M11" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="N11" t="s">
-        <v>167</v>
+        <v>143</v>
       </c>
       <c r="O11">
         <v>3</v>
       </c>
       <c r="P11" t="s">
-        <v>168</v>
+        <v>144</v>
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.2">
@@ -3251,16 +3179,16 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>75</v>
+        <v>63</v>
       </c>
       <c r="C12" t="s">
-        <v>76</v>
+        <v>64</v>
       </c>
       <c r="D12" t="s">
-        <v>77</v>
+        <v>65</v>
       </c>
       <c r="E12" t="s">
-        <v>169</v>
+        <v>145</v>
       </c>
       <c r="F12">
         <v>12831</v>
@@ -3282,19 +3210,19 @@
         <v>1.194887912E-2</v>
       </c>
       <c r="L12" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="M12" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="N12" t="s">
-        <v>170</v>
+        <v>146</v>
       </c>
       <c r="O12">
         <v>10</v>
       </c>
       <c r="P12" t="s">
-        <v>171</v>
+        <v>147</v>
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.2">
@@ -3302,16 +3230,16 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>75</v>
+        <v>63</v>
       </c>
       <c r="C13" t="s">
-        <v>81</v>
+        <v>69</v>
       </c>
       <c r="D13" t="s">
-        <v>82</v>
+        <v>70</v>
       </c>
       <c r="E13" t="s">
-        <v>172</v>
+        <v>148</v>
       </c>
       <c r="F13">
         <v>11779</v>
@@ -3333,19 +3261,19 @@
         <v>1.442530356E-2</v>
       </c>
       <c r="L13" t="s">
-        <v>72</v>
+        <v>60</v>
       </c>
       <c r="M13" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="N13" t="s">
-        <v>173</v>
+        <v>149</v>
       </c>
       <c r="O13">
         <v>8</v>
       </c>
       <c r="P13" t="s">
-        <v>174</v>
+        <v>150</v>
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.2">
@@ -3353,16 +3281,16 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
+        <v>63</v>
+      </c>
+      <c r="C14" t="s">
+        <v>74</v>
+      </c>
+      <c r="D14" t="s">
         <v>75</v>
       </c>
-      <c r="C14" t="s">
-        <v>86</v>
-      </c>
-      <c r="D14" t="s">
-        <v>87</v>
-      </c>
       <c r="E14" t="s">
-        <v>175</v>
+        <v>151</v>
       </c>
       <c r="F14">
         <v>4450</v>
@@ -3384,19 +3312,19 @@
         <v>1.168629472E-2</v>
       </c>
       <c r="L14" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="M14" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="N14" t="s">
-        <v>176</v>
+        <v>152</v>
       </c>
       <c r="O14">
         <v>10</v>
       </c>
       <c r="P14" t="s">
-        <v>177</v>
+        <v>153</v>
       </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.2">
@@ -3404,16 +3332,16 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>75</v>
+        <v>63</v>
       </c>
       <c r="C15" t="s">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="D15" t="s">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="E15" t="s">
-        <v>178</v>
+        <v>154</v>
       </c>
       <c r="F15">
         <v>16751</v>
@@ -3435,19 +3363,19 @@
         <v>1.264529853E-2</v>
       </c>
       <c r="L15" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="M15" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="N15" t="s">
-        <v>179</v>
+        <v>155</v>
       </c>
       <c r="O15">
         <v>8</v>
       </c>
       <c r="P15" t="s">
-        <v>180</v>
+        <v>156</v>
       </c>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.2">
@@ -3455,16 +3383,16 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>96</v>
+        <v>84</v>
       </c>
       <c r="C16" t="s">
-        <v>97</v>
+        <v>85</v>
       </c>
       <c r="D16" t="s">
-        <v>98</v>
+        <v>86</v>
       </c>
       <c r="E16" t="s">
-        <v>181</v>
+        <v>157</v>
       </c>
       <c r="F16">
         <v>60144</v>
@@ -3486,19 +3414,19 @@
         <v>1.7605521919999999E-2</v>
       </c>
       <c r="L16" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="M16" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="N16" t="s">
-        <v>182</v>
+        <v>158</v>
       </c>
       <c r="O16">
         <v>0</v>
       </c>
       <c r="P16" t="s">
-        <v>183</v>
+        <v>159</v>
       </c>
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.2">
@@ -3506,16 +3434,16 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>96</v>
+        <v>84</v>
       </c>
       <c r="C17" t="s">
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="D17" t="s">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="E17" t="s">
-        <v>184</v>
+        <v>160</v>
       </c>
       <c r="F17">
         <v>7213</v>
@@ -3537,19 +3465,19 @@
         <v>1.4850037470000001E-2</v>
       </c>
       <c r="L17" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="M17" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="N17" t="s">
-        <v>185</v>
+        <v>161</v>
       </c>
       <c r="O17">
         <v>8</v>
       </c>
       <c r="P17" t="s">
-        <v>186</v>
+        <v>162</v>
       </c>
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.2">
@@ -3557,16 +3485,16 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
+        <v>84</v>
+      </c>
+      <c r="C18" t="s">
+        <v>95</v>
+      </c>
+      <c r="D18" t="s">
         <v>96</v>
       </c>
-      <c r="C18" t="s">
-        <v>107</v>
-      </c>
-      <c r="D18" t="s">
-        <v>108</v>
-      </c>
       <c r="E18" t="s">
-        <v>187</v>
+        <v>163</v>
       </c>
       <c r="F18">
         <v>53423</v>
@@ -3588,19 +3516,19 @@
         <v>1.731289242E-2</v>
       </c>
       <c r="L18" t="s">
-        <v>72</v>
+        <v>60</v>
       </c>
       <c r="M18" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="N18" t="s">
-        <v>188</v>
+        <v>164</v>
       </c>
       <c r="O18">
         <v>8</v>
       </c>
       <c r="P18" t="s">
-        <v>189</v>
+        <v>165</v>
       </c>
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.2">
@@ -3608,16 +3536,16 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>96</v>
+        <v>84</v>
       </c>
       <c r="C19" t="s">
-        <v>112</v>
+        <v>100</v>
       </c>
       <c r="D19" t="s">
-        <v>113</v>
+        <v>101</v>
       </c>
       <c r="E19" t="s">
-        <v>190</v>
+        <v>166</v>
       </c>
       <c r="F19">
         <v>55314</v>
@@ -3639,19 +3567,19 @@
         <v>1.435039418E-2</v>
       </c>
       <c r="L19" t="s">
-        <v>191</v>
+        <v>167</v>
       </c>
       <c r="M19" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="N19" t="s">
-        <v>192</v>
+        <v>168</v>
       </c>
       <c r="O19">
         <v>8</v>
       </c>
       <c r="P19" t="s">
-        <v>193</v>
+        <v>169</v>
       </c>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.2">
@@ -3659,16 +3587,16 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>117</v>
+        <v>105</v>
       </c>
       <c r="C20" t="s">
-        <v>118</v>
+        <v>106</v>
       </c>
       <c r="D20" t="s">
-        <v>119</v>
+        <v>107</v>
       </c>
       <c r="E20" t="s">
-        <v>194</v>
+        <v>170</v>
       </c>
       <c r="F20">
         <v>147511</v>
@@ -3690,19 +3618,19 @@
         <v>1.6941747930000001E-2</v>
       </c>
       <c r="L20" t="s">
-        <v>195</v>
+        <v>171</v>
       </c>
       <c r="M20" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="N20" t="s">
-        <v>196</v>
+        <v>172</v>
       </c>
       <c r="O20">
         <v>3</v>
       </c>
       <c r="P20" t="s">
-        <v>197</v>
+        <v>173</v>
       </c>
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.2">
@@ -3710,16 +3638,16 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>117</v>
+        <v>105</v>
       </c>
       <c r="C21" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
       <c r="D21" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="E21" t="s">
-        <v>198</v>
+        <v>174</v>
       </c>
       <c r="F21">
         <v>4692</v>
@@ -3741,19 +3669,19 @@
         <v>1.495814887E-2</v>
       </c>
       <c r="L21" t="s">
-        <v>199</v>
+        <v>175</v>
       </c>
       <c r="M21" t="s">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="N21" t="s">
-        <v>200</v>
+        <v>176</v>
       </c>
       <c r="O21">
         <v>2</v>
       </c>
       <c r="P21" t="s">
-        <v>201</v>
+        <v>177</v>
       </c>
     </row>
   </sheetData>
@@ -3766,6 +3694,8 @@
   <dimension ref="A1:Q21"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="255.7109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="19.7109375" customWidth="1"/>
     <col min="7" max="7" width="22.28515625" customWidth="1"/>
   </cols>
@@ -3784,43 +3714,43 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>202</v>
+        <v>237</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>203</v>
+        <v>238</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>204</v>
+        <v>239</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>205</v>
+        <v>240</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>206</v>
+        <v>241</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>207</v>
+        <v>242</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>208</v>
+        <v>249</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>209</v>
+        <v>243</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>210</v>
+        <v>244</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>211</v>
+        <v>245</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>212</v>
+        <v>246</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>213</v>
+        <v>247</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>214</v>
+        <v>248</v>
       </c>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.2">
@@ -3828,16 +3758,16 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="D2" t="s">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="E2" t="s">
-        <v>215</v>
+        <v>178</v>
       </c>
       <c r="F2">
         <v>7108</v>
@@ -3862,19 +3792,19 @@
         <v>141047.00080000001</v>
       </c>
       <c r="M2" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="N2" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="O2" t="s">
-        <v>216</v>
+        <v>179</v>
       </c>
       <c r="P2">
         <v>8</v>
       </c>
       <c r="Q2" t="s">
-        <v>217</v>
+        <v>180</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.2">
@@ -3882,16 +3812,16 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="C3" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="D3" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="E3" t="s">
-        <v>218</v>
+        <v>181</v>
       </c>
       <c r="F3">
         <v>7113</v>
@@ -3916,19 +3846,19 @@
         <v>141047.0007</v>
       </c>
       <c r="M3" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="N3" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="O3" t="s">
-        <v>219</v>
+        <v>182</v>
       </c>
       <c r="P3">
         <v>8</v>
       </c>
       <c r="Q3" t="s">
-        <v>220</v>
+        <v>183</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.2">
@@ -3936,16 +3866,16 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="C4" t="s">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="D4" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="E4" t="s">
-        <v>221</v>
+        <v>184</v>
       </c>
       <c r="F4">
         <v>5551</v>
@@ -3970,19 +3900,19 @@
         <v>141047.0007</v>
       </c>
       <c r="M4" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="N4" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="O4" t="s">
-        <v>222</v>
+        <v>185</v>
       </c>
       <c r="P4">
         <v>10</v>
       </c>
       <c r="Q4" t="s">
-        <v>223</v>
+        <v>186</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.2">
@@ -3990,16 +3920,16 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="C5" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="D5" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="E5" t="s">
-        <v>224</v>
+        <v>187</v>
       </c>
       <c r="F5">
         <v>9212</v>
@@ -4024,19 +3954,19 @@
         <v>141047.00080000001</v>
       </c>
       <c r="M5" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="N5" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="O5" t="s">
-        <v>225</v>
+        <v>188</v>
       </c>
       <c r="P5">
         <v>8</v>
       </c>
       <c r="Q5" t="s">
-        <v>226</v>
+        <v>189</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.2">
@@ -4044,16 +3974,16 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" t="s">
         <v>29</v>
       </c>
-      <c r="C6" t="s">
-        <v>40</v>
-      </c>
-      <c r="D6" t="s">
-        <v>41</v>
-      </c>
       <c r="E6" t="s">
-        <v>227</v>
+        <v>190</v>
       </c>
       <c r="F6">
         <v>8375</v>
@@ -4078,19 +4008,19 @@
         <v>141047.0007</v>
       </c>
       <c r="M6" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="N6" t="s">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="O6" t="s">
-        <v>228</v>
+        <v>191</v>
       </c>
       <c r="P6">
         <v>2</v>
       </c>
       <c r="Q6" t="s">
-        <v>229</v>
+        <v>192</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.2">
@@ -4098,16 +4028,16 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="C7" t="s">
-        <v>47</v>
+        <v>35</v>
       </c>
       <c r="D7" t="s">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="E7" t="s">
-        <v>230</v>
+        <v>193</v>
       </c>
       <c r="F7">
         <v>9057</v>
@@ -4132,19 +4062,19 @@
         <v>141047.00099999999</v>
       </c>
       <c r="M7" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="N7" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="O7" t="s">
-        <v>231</v>
+        <v>194</v>
       </c>
       <c r="P7">
         <v>8</v>
       </c>
       <c r="Q7" t="s">
-        <v>232</v>
+        <v>195</v>
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.2">
@@ -4152,16 +4082,16 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>52</v>
+        <v>40</v>
       </c>
       <c r="C8" t="s">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="D8" t="s">
-        <v>54</v>
+        <v>42</v>
       </c>
       <c r="E8" t="s">
-        <v>233</v>
+        <v>196</v>
       </c>
       <c r="F8">
         <v>6598</v>
@@ -4186,19 +4116,19 @@
         <v>141047.00039999999</v>
       </c>
       <c r="M8" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="N8" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="O8" t="s">
-        <v>234</v>
+        <v>197</v>
       </c>
       <c r="P8">
         <v>4</v>
       </c>
       <c r="Q8" t="s">
-        <v>235</v>
+        <v>198</v>
       </c>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.2">
@@ -4206,16 +4136,16 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>52</v>
+        <v>40</v>
       </c>
       <c r="C9" t="s">
-        <v>59</v>
+        <v>47</v>
       </c>
       <c r="D9" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="E9" t="s">
-        <v>236</v>
+        <v>199</v>
       </c>
       <c r="F9">
         <v>4623</v>
@@ -4240,19 +4170,19 @@
         <v>141047.00049999999</v>
       </c>
       <c r="M9" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="N9" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="O9" t="s">
-        <v>237</v>
+        <v>200</v>
       </c>
       <c r="P9">
         <v>10</v>
       </c>
       <c r="Q9" t="s">
-        <v>238</v>
+        <v>201</v>
       </c>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.2">
@@ -4260,16 +4190,16 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
+        <v>40</v>
+      </c>
+      <c r="C10" t="s">
+        <v>51</v>
+      </c>
+      <c r="D10" t="s">
         <v>52</v>
       </c>
-      <c r="C10" t="s">
-        <v>63</v>
-      </c>
-      <c r="D10" t="s">
-        <v>64</v>
-      </c>
       <c r="E10" t="s">
-        <v>239</v>
+        <v>202</v>
       </c>
       <c r="F10">
         <v>12280</v>
@@ -4294,19 +4224,19 @@
         <v>141047.00090000001</v>
       </c>
       <c r="M10" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="N10" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="O10" t="s">
-        <v>240</v>
+        <v>203</v>
       </c>
       <c r="P10">
         <v>8</v>
       </c>
       <c r="Q10" t="s">
-        <v>241</v>
+        <v>204</v>
       </c>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.2">
@@ -4314,16 +4244,16 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>52</v>
+        <v>40</v>
       </c>
       <c r="C11" t="s">
-        <v>69</v>
+        <v>57</v>
       </c>
       <c r="D11" t="s">
-        <v>70</v>
+        <v>58</v>
       </c>
       <c r="E11" t="s">
-        <v>242</v>
+        <v>205</v>
       </c>
       <c r="F11">
         <v>7635</v>
@@ -4348,19 +4278,19 @@
         <v>141047.00039999999</v>
       </c>
       <c r="M11" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="N11" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="O11" t="s">
-        <v>243</v>
+        <v>206</v>
       </c>
       <c r="P11">
         <v>3</v>
       </c>
       <c r="Q11" t="s">
-        <v>244</v>
+        <v>207</v>
       </c>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.2">
@@ -4368,16 +4298,16 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>75</v>
+        <v>63</v>
       </c>
       <c r="C12" t="s">
-        <v>76</v>
+        <v>64</v>
       </c>
       <c r="D12" t="s">
-        <v>77</v>
+        <v>65</v>
       </c>
       <c r="E12" t="s">
-        <v>245</v>
+        <v>208</v>
       </c>
       <c r="F12">
         <v>8483</v>
@@ -4402,19 +4332,19 @@
         <v>141047.0007</v>
       </c>
       <c r="M12" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="N12" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="O12" t="s">
-        <v>246</v>
+        <v>209</v>
       </c>
       <c r="P12">
         <v>9</v>
       </c>
       <c r="Q12" t="s">
-        <v>247</v>
+        <v>210</v>
       </c>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.2">
@@ -4422,16 +4352,16 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>75</v>
+        <v>63</v>
       </c>
       <c r="C13" t="s">
-        <v>81</v>
+        <v>69</v>
       </c>
       <c r="D13" t="s">
-        <v>82</v>
+        <v>70</v>
       </c>
       <c r="E13" t="s">
-        <v>248</v>
+        <v>211</v>
       </c>
       <c r="F13">
         <v>18614</v>
@@ -4456,19 +4386,19 @@
         <v>141047.00150000001</v>
       </c>
       <c r="M13" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="N13" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="O13" t="s">
-        <v>249</v>
+        <v>212</v>
       </c>
       <c r="P13">
         <v>8</v>
       </c>
       <c r="Q13" t="s">
-        <v>250</v>
+        <v>213</v>
       </c>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.2">
@@ -4476,16 +4406,16 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
+        <v>63</v>
+      </c>
+      <c r="C14" t="s">
+        <v>74</v>
+      </c>
+      <c r="D14" t="s">
         <v>75</v>
       </c>
-      <c r="C14" t="s">
-        <v>86</v>
-      </c>
-      <c r="D14" t="s">
-        <v>87</v>
-      </c>
       <c r="E14" t="s">
-        <v>251</v>
+        <v>214</v>
       </c>
       <c r="F14">
         <v>6051</v>
@@ -4510,19 +4440,19 @@
         <v>141047.00049999999</v>
       </c>
       <c r="M14" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="N14" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="O14" t="s">
-        <v>176</v>
+        <v>152</v>
       </c>
       <c r="P14">
         <v>10</v>
       </c>
       <c r="Q14" t="s">
-        <v>252</v>
+        <v>215</v>
       </c>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.2">
@@ -4530,16 +4460,16 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>75</v>
+        <v>63</v>
       </c>
       <c r="C15" t="s">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="D15" t="s">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="E15" t="s">
-        <v>253</v>
+        <v>216</v>
       </c>
       <c r="F15">
         <v>8849</v>
@@ -4564,19 +4494,19 @@
         <v>141047.0007</v>
       </c>
       <c r="M15" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="N15" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="O15" t="s">
-        <v>254</v>
+        <v>217</v>
       </c>
       <c r="P15">
         <v>8</v>
       </c>
       <c r="Q15" t="s">
-        <v>255</v>
+        <v>218</v>
       </c>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.2">
@@ -4584,16 +4514,16 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>96</v>
+        <v>84</v>
       </c>
       <c r="C16" t="s">
-        <v>97</v>
+        <v>85</v>
       </c>
       <c r="D16" t="s">
-        <v>98</v>
+        <v>86</v>
       </c>
       <c r="E16" t="s">
-        <v>256</v>
+        <v>219</v>
       </c>
       <c r="F16">
         <v>8785</v>
@@ -4618,19 +4548,19 @@
         <v>141047.0007</v>
       </c>
       <c r="M16" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="N16" t="s">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="O16" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="P16">
         <v>6</v>
       </c>
       <c r="Q16" t="s">
-        <v>258</v>
+        <v>221</v>
       </c>
     </row>
     <row r="17" spans="1:17" x14ac:dyDescent="0.2">
@@ -4638,16 +4568,16 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>96</v>
+        <v>84</v>
       </c>
       <c r="C17" t="s">
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="D17" t="s">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="E17" t="s">
-        <v>259</v>
+        <v>222</v>
       </c>
       <c r="F17">
         <v>10522</v>
@@ -4672,19 +4602,19 @@
         <v>141047.0007</v>
       </c>
       <c r="M17" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="N17" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="O17" t="s">
-        <v>260</v>
+        <v>223</v>
       </c>
       <c r="P17">
         <v>6</v>
       </c>
       <c r="Q17" t="s">
-        <v>261</v>
+        <v>224</v>
       </c>
     </row>
     <row r="18" spans="1:17" x14ac:dyDescent="0.2">
@@ -4692,16 +4622,16 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
+        <v>84</v>
+      </c>
+      <c r="C18" t="s">
+        <v>95</v>
+      </c>
+      <c r="D18" t="s">
         <v>96</v>
       </c>
-      <c r="C18" t="s">
-        <v>107</v>
-      </c>
-      <c r="D18" t="s">
-        <v>108</v>
-      </c>
       <c r="E18" t="s">
-        <v>262</v>
+        <v>225</v>
       </c>
       <c r="F18">
         <v>11106</v>
@@ -4726,19 +4656,19 @@
         <v>141047.00099999999</v>
       </c>
       <c r="M18" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="N18" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="O18" t="s">
-        <v>263</v>
+        <v>226</v>
       </c>
       <c r="P18">
         <v>8</v>
       </c>
       <c r="Q18" t="s">
-        <v>264</v>
+        <v>227</v>
       </c>
     </row>
     <row r="19" spans="1:17" x14ac:dyDescent="0.2">
@@ -4746,16 +4676,16 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>96</v>
+        <v>84</v>
       </c>
       <c r="C19" t="s">
-        <v>112</v>
+        <v>100</v>
       </c>
       <c r="D19" t="s">
-        <v>113</v>
+        <v>101</v>
       </c>
       <c r="E19" t="s">
-        <v>265</v>
+        <v>228</v>
       </c>
       <c r="F19">
         <v>7463</v>
@@ -4780,19 +4710,19 @@
         <v>141047.0007</v>
       </c>
       <c r="M19" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="N19" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="O19" t="s">
-        <v>266</v>
+        <v>229</v>
       </c>
       <c r="P19">
         <v>8</v>
       </c>
       <c r="Q19" t="s">
-        <v>267</v>
+        <v>230</v>
       </c>
     </row>
     <row r="20" spans="1:17" x14ac:dyDescent="0.2">
@@ -4800,16 +4730,16 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>117</v>
+        <v>105</v>
       </c>
       <c r="C20" t="s">
-        <v>118</v>
+        <v>106</v>
       </c>
       <c r="D20" t="s">
-        <v>119</v>
+        <v>107</v>
       </c>
       <c r="E20" t="s">
-        <v>268</v>
+        <v>231</v>
       </c>
       <c r="F20">
         <v>12691</v>
@@ -4834,19 +4764,19 @@
         <v>141047.00080000001</v>
       </c>
       <c r="M20" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="N20" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="O20" t="s">
-        <v>269</v>
+        <v>232</v>
       </c>
       <c r="P20">
         <v>5</v>
       </c>
       <c r="Q20" t="s">
-        <v>270</v>
+        <v>233</v>
       </c>
     </row>
     <row r="21" spans="1:17" x14ac:dyDescent="0.2">
@@ -4854,16 +4784,16 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>117</v>
+        <v>105</v>
       </c>
       <c r="C21" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
       <c r="D21" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="E21" t="s">
-        <v>271</v>
+        <v>234</v>
       </c>
       <c r="F21">
         <v>11097</v>
@@ -4888,19 +4818,19 @@
         <v>141047.0007</v>
       </c>
       <c r="M21" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="N21" t="s">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="O21" t="s">
-        <v>272</v>
+        <v>235</v>
       </c>
       <c r="P21">
         <v>10</v>
       </c>
       <c r="Q21" t="s">
-        <v>273</v>
+        <v>236</v>
       </c>
     </row>
   </sheetData>

</xml_diff>